<commit_message>
Polish form demos and fetch form fonts from Google Fonts
</commit_message>
<xml_diff>
--- a/converter/xlsx/testdata/form-fixed.xlsx
+++ b/converter/xlsx/testdata/form-fixed.xlsx
@@ -478,7 +478,7 @@
     <row r="1" ht="27" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>明書 Certificate</t>
+          <t>明細書 Certificate</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -623,11 +623,6 @@
       <c r="A15" t="inlineStr">
         <is>
           <t>{{missing}}</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>\{{not a tag}}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Polish form demos and fetch form fonts from Google Fonts (#92)
</commit_message>
<xml_diff>
--- a/converter/xlsx/testdata/form-fixed.xlsx
+++ b/converter/xlsx/testdata/form-fixed.xlsx
@@ -478,7 +478,7 @@
     <row r="1" ht="27" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>明書 Certificate</t>
+          <t>明細書 Certificate</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -623,11 +623,6 @@
       <c r="A15" t="inlineStr">
         <is>
           <t>{{missing}}</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>\{{not a tag}}</t>
         </is>
       </c>
     </row>

</xml_diff>